<commit_message>
Add user input for number of games and suggestions; enhance suggestion logic
</commit_message>
<xml_diff>
--- a/src/sugestoes_mega_sena.xlsx
+++ b/src/sugestoes_mega_sena.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -448,7 +448,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>7, 9, 22, 31, 48, 55</t>
+          <t>7, 12, 18, 21, 22, 31, 58</t>
         </is>
       </c>
     </row>
@@ -460,19 +460,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>9, 12, 21, 22, 31, 40</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Sugestão 3</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>3, 9, 21, 22, 40, 48</t>
+          <t>3, 7, 12, 15, 26, 40, 48</t>
         </is>
       </c>
     </row>

</xml_diff>